<commit_message>
update Sapporo - Otaru
</commit_message>
<xml_diff>
--- a/travel/삿포로/2026_삿포로.xlsx
+++ b/travel/삿포로/2026_삿포로.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\csw\travel\삿포로\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\csw\travel\삿포로\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C3B55F-26C0-408A-B54B-F91A235A8D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC4B876-A67E-4334-B919-0F3B5957CF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{16BD92D5-DB44-4AB7-83A8-7317C0E10327}"/>
+    <workbookView xWindow="28680" yWindow="4500" windowWidth="29040" windowHeight="15720" xr2:uid="{16BD92D5-DB44-4AB7-83A8-7317C0E10327}"/>
   </bookViews>
   <sheets>
     <sheet name="일정" sheetId="2" r:id="rId1"/>
@@ -34,15 +34,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>일</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -196,10 +193,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>점심식사(준페이식당)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>청의호수</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -221,6 +214,37 @@
   </si>
   <si>
     <t>점심</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스스키노 -&gt; 삿포로 역
+(지하철)
+삿포로 역 -&gt; 미나미 오타루
+(JR 열차 자유석)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점심식사
+(준페이식당)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[시카이마치도리 거리]
+오르골당
+증기 시계
+기타이치 유리 3호관
+르타오 무료전망대
+(치즈케이크)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오타루 운하
+오타루 삼각시장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점심
+(스시거리 or 삼각시장 - 카이센동)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -596,13 +620,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -644,15 +668,6 @@
     <xf numFmtId="20" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -663,9 +678,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -712,6 +724,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1778,7 +1802,9 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="25.625" customWidth="1"/>
+    <col min="3" max="3" width="25.625" customWidth="1"/>
+    <col min="4" max="4" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="25.625" customWidth="1"/>
     <col min="10" max="10" width="15.875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="42.125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1819,73 +1845,73 @@
       <c r="B4" s="6">
         <v>0</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="6">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="6">
         <v>8.3333333333333301E-2</v>
       </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="6">
         <v>0.125</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
         <v>0.16666666666666699</v>
       </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="46"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="6">
         <v>0.20833333333333301</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="6">
         <v>0.25</v>
       </c>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="6">
         <v>0.29166666666666702</v>
       </c>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="2:8" ht="33" x14ac:dyDescent="0.3">
       <c r="B12" s="6">
@@ -1897,29 +1923,33 @@
       <c r="D12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="44" t="s">
+      <c r="E12" s="40" t="s">
         <v>23</v>
       </c>
       <c r="F12" s="7"/>
     </row>
-    <row r="13" spans="2:8" ht="33" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="66" x14ac:dyDescent="0.3">
       <c r="B13" s="6">
         <v>0.375</v>
       </c>
       <c r="C13" s="22"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="45" t="s">
+      <c r="D13" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="41" t="s">
         <v>34</v>
       </c>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="99" x14ac:dyDescent="0.3">
       <c r="B14" s="6">
         <v>0.41666666666666702</v>
       </c>
       <c r="C14" s="22"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="44" t="s">
+      <c r="D14" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="40" t="s">
         <v>35</v>
       </c>
       <c r="F14" s="7"/>
@@ -1932,23 +1962,23 @@
         <v>6</v>
       </c>
       <c r="D15" s="7"/>
-      <c r="E15" s="45" t="s">
+      <c r="E15" s="41" t="s">
         <v>36</v>
       </c>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="2:8" ht="33" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B16" s="6">
         <v>0.5</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="44" t="s">
-        <v>37</v>
+        <v>42</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>44</v>
       </c>
       <c r="F16" s="21" t="s">
         <v>7</v>
@@ -1960,21 +1990,23 @@
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="44" t="s">
-        <v>38</v>
+      <c r="E17" s="40" t="s">
+        <v>37</v>
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" ht="33" x14ac:dyDescent="0.3">
       <c r="B18" s="6">
         <v>0.58333333333333304</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="44" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>38</v>
       </c>
       <c r="F18" s="22"/>
     </row>
@@ -1984,8 +2016,8 @@
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
-      <c r="E19" s="44" t="s">
-        <v>40</v>
+      <c r="E19" s="40" t="s">
+        <v>39</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>8</v>
@@ -1997,7 +2029,7 @@
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
-      <c r="E20" s="44" t="s">
+      <c r="E20" s="40" t="s">
         <v>35</v>
       </c>
       <c r="F20" s="7"/>
@@ -2008,7 +2040,7 @@
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
-      <c r="E21" s="44"/>
+      <c r="E21" s="40"/>
       <c r="F21" s="7"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
@@ -2021,7 +2053,7 @@
       <c r="D22" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="44"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="7"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
@@ -2030,7 +2062,7 @@
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
-      <c r="E23" s="44"/>
+      <c r="E23" s="40"/>
       <c r="F23" s="7"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
@@ -2039,8 +2071,8 @@
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
-      <c r="E24" s="44" t="s">
-        <v>41</v>
+      <c r="E24" s="40" t="s">
+        <v>40</v>
       </c>
       <c r="F24" s="7"/>
     </row>
@@ -2075,11 +2107,11 @@
       <c r="B28" s="23">
         <v>1</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="25"/>
-      <c r="E28" s="26"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="45"/>
       <c r="F28" s="17"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
@@ -2103,6 +2135,9 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Internal</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -2127,6 +2162,9 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Internal</oddFooter>
+  </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -2143,474 +2181,474 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="32"/>
-      <c r="C2" s="32" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="E2" s="31"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="33">
+      <c r="C3" s="29">
         <v>1</v>
       </c>
-      <c r="D3" s="33">
+      <c r="D3" s="29">
         <v>8.6265999999999998</v>
       </c>
-      <c r="E3" s="31"/>
+      <c r="E3" s="8"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="35">
+      <c r="C4" s="31">
         <f>681900*2</f>
         <v>1363800</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="35">
+      <c r="C5" s="31">
         <v>472602</v>
       </c>
-      <c r="D5" s="35"/>
-      <c r="E5" s="36"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="32"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="35">
+      <c r="C6" s="31">
         <f>57000*2</f>
         <v>114000</v>
       </c>
-      <c r="D6" s="35"/>
-      <c r="E6" s="36"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="32"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="34"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="36"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="37"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="36"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="32"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="38"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="34"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="32"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="38"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="36"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="32"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="37"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="34"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="34"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="32"/>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="32"/>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="34"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="36"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="32"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" s="34"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" s="34"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="36"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="34"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="36"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="32"/>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="34"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="32"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="34"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="32"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="34"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="32"/>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" s="34"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="32"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="34"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="32"/>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="34"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="32"/>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="34"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32"/>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B28" s="34"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32"/>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B29" s="34"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="36"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B30" s="34"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="32"/>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B31" s="34"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="36"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="32"/>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B32" s="34"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="36"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="32"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B33" s="34"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="36"/>
+      <c r="B33" s="30"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B34" s="34"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="32"/>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B35" s="34"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="36"/>
+      <c r="B35" s="30"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="32"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B36" s="34"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="36"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B37" s="34"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="36"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B38" s="34"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="32"/>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B39" s="34"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="36"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="32"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B40" s="34"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="36"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="32"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B41" s="34"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="36"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="32"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B42" s="34"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="36"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="32"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B43" s="34"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="36"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="32"/>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B44" s="34"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="36"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="32"/>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B45" s="34"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="36"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="32"/>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B46" s="34"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="36"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="32"/>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B47" s="34"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="36"/>
+      <c r="B47" s="30"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="32"/>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B48" s="34"/>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="36"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="32"/>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B49" s="34"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="36"/>
+      <c r="B49" s="30"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="32"/>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B50" s="34"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="36"/>
+      <c r="B50" s="30"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="31"/>
+      <c r="E50" s="32"/>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B51" s="34"/>
-      <c r="C51" s="35"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="36"/>
+      <c r="B51" s="30"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="32"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B52" s="34"/>
-      <c r="C52" s="35"/>
-      <c r="D52" s="35"/>
-      <c r="E52" s="36"/>
+      <c r="B52" s="30"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="31"/>
+      <c r="E52" s="32"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B53" s="34"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="36"/>
+      <c r="B53" s="30"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="32"/>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B54" s="34"/>
-      <c r="C54" s="35"/>
-      <c r="D54" s="35"/>
-      <c r="E54" s="36"/>
+      <c r="B54" s="30"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="31"/>
+      <c r="E54" s="32"/>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B55" s="34"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="36"/>
+      <c r="B55" s="30"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="31"/>
+      <c r="E55" s="32"/>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B56" s="34"/>
-      <c r="C56" s="35"/>
-      <c r="D56" s="35"/>
-      <c r="E56" s="36"/>
+      <c r="B56" s="30"/>
+      <c r="C56" s="31"/>
+      <c r="D56" s="31"/>
+      <c r="E56" s="32"/>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B57" s="34"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="36"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="32"/>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B58" s="34"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="36"/>
+      <c r="B58" s="30"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="31"/>
+      <c r="E58" s="32"/>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B59" s="34"/>
-      <c r="C59" s="35"/>
-      <c r="D59" s="35"/>
-      <c r="E59" s="36"/>
+      <c r="B59" s="30"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="31"/>
+      <c r="E59" s="32"/>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B60" s="34"/>
-      <c r="C60" s="35"/>
-      <c r="D60" s="35"/>
-      <c r="E60" s="36"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="31"/>
+      <c r="E60" s="32"/>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B61" s="34"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="35"/>
-      <c r="E61" s="36"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="31"/>
+      <c r="D61" s="31"/>
+      <c r="E61" s="32"/>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B62" s="34"/>
-      <c r="C62" s="35"/>
-      <c r="D62" s="35"/>
-      <c r="E62" s="36"/>
+      <c r="B62" s="30"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="31"/>
+      <c r="E62" s="32"/>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B63" s="34"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="35"/>
-      <c r="E63" s="36"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="32"/>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B64" s="34"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="36"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="31"/>
+      <c r="E64" s="32"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B65" s="34"/>
-      <c r="C65" s="35"/>
-      <c r="D65" s="35"/>
-      <c r="E65" s="36"/>
+      <c r="B65" s="30"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="E65" s="32"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B66" s="34"/>
-      <c r="C66" s="35"/>
-      <c r="D66" s="35"/>
-      <c r="E66" s="36"/>
+      <c r="B66" s="30"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="E66" s="32"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B67" s="34"/>
-      <c r="C67" s="35"/>
-      <c r="D67" s="35"/>
-      <c r="E67" s="36"/>
+      <c r="B67" s="30"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="32"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B68" s="34"/>
-      <c r="C68" s="35"/>
-      <c r="D68" s="35"/>
-      <c r="E68" s="36"/>
+      <c r="B68" s="30"/>
+      <c r="C68" s="31"/>
+      <c r="D68" s="31"/>
+      <c r="E68" s="32"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B69" s="34"/>
-      <c r="C69" s="35"/>
-      <c r="D69" s="35"/>
-      <c r="E69" s="36"/>
+      <c r="B69" s="30"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="32"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B70" s="34"/>
-      <c r="C70" s="35"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="36"/>
+      <c r="B70" s="30"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="32"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B71" s="34"/>
-      <c r="C71" s="35"/>
-      <c r="D71" s="35"/>
-      <c r="E71" s="36"/>
+      <c r="B71" s="30"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="31"/>
+      <c r="E71" s="32"/>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B72" s="34"/>
-      <c r="C72" s="35"/>
-      <c r="D72" s="35"/>
-      <c r="E72" s="36"/>
+      <c r="B72" s="30"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="32"/>
     </row>
     <row r="73" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B73" s="39"/>
-      <c r="C73" s="40"/>
-      <c r="D73" s="40"/>
-      <c r="E73" s="36"/>
+      <c r="B73" s="35"/>
+      <c r="C73" s="36"/>
+      <c r="D73" s="36"/>
+      <c r="E73" s="32"/>
     </row>
     <row r="74" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="41" t="s">
+      <c r="B74" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C74" s="42">
+      <c r="C74" s="38">
         <f>SUM(C4:C73)*C3</f>
         <v>1950402</v>
       </c>
-      <c r="D74" s="42">
+      <c r="D74" s="38">
         <f>SUM(D4:D73)*D3</f>
         <v>0</v>
       </c>
-      <c r="E74" s="43">
+      <c r="E74" s="39">
         <f>SUM(C74:D74)</f>
         <v>1950402</v>
       </c>
@@ -2618,6 +2656,9 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Internal</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -2684,19 +2725,19 @@
       </c>
     </row>
     <row r="5" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="27">
+      <c r="B5" s="24">
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="26">
         <v>190497</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="27">
         <v>1</v>
       </c>
     </row>
@@ -2726,6 +2767,15 @@
     <hyperlink ref="C6" r:id="rId4" xr:uid="{008F70B1-1F63-445B-AC47-BF60217FFFC7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Internal</oddFooter>
+  </headerFooter>
   <drawing r:id="rId5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7e753c2c-bb14-4786-921b-97c6a6fc424f}" enabled="1" method="Standard" siteId="{3bd97919-57c3-48d3-9e9a-8e4c01614a8f}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>